<commit_message>
fix(excel): inject cache-busting timestamp to download url to prevent browser caching stale files
</commit_message>
<xml_diff>
--- a/storage/upload/hasil_mcu_program (Daesang)-NEW2.xlsx
+++ b/storage/upload/hasil_mcu_program (Daesang)-NEW2.xlsx
@@ -489,11 +489,7 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1998-12-20 00:00:00</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-30 00:00:00</t>
@@ -532,11 +528,7 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1987-06-11 00:00:00</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-30 00:00:00</t>
@@ -575,11 +567,7 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1988-10-21 00:00:00</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2026-06-30 00:00:00</t>
@@ -618,11 +606,7 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1994-11-01 00:00:00</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-06-30 00:00:00</t>
@@ -663,7 +647,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2000-03-11 00:00:00</t>
+          <t>1987-06-11 00:00:00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -706,7 +690,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1997-03-05 00:00:00</t>
+          <t>1988-10-21 00:00:00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -749,7 +733,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1998-01-10 00:00:00</t>
+          <t>1997-04-17 00:00:00</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -792,7 +776,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1996-01-13 00:00:00</t>
+          <t>1999-12-02 00:00:00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -835,7 +819,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1997-04-17 00:00:00</t>
+          <t>1992-07-02 00:00:00</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -878,7 +862,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1999-12-02 00:00:00</t>
+          <t>1982-09-17 00:00:00</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -921,7 +905,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2003-03-02 00:00:00</t>
+          <t>1998-07-05 00:00:00</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -964,7 +948,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1991-07-21 00:00:00</t>
+          <t>2000-04-25 00:00:00</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1007,7 +991,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1998-07-12 00:00:00</t>
+          <t>2002-10-27 00:00:00</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1050,7 +1034,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1992-07-02 00:00:00</t>
+          <t>1997-11-14 00:00:00</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1093,7 +1077,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1982-09-17 00:00:00</t>
+          <t>1994-09-04 00:00:00</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1136,7 +1120,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1994-08-14 00:00:00</t>
+          <t>1998-12-20 00:00:00</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1179,7 +1163,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1995-06-13 00:00:00</t>
+          <t>1994-11-01 00:00:00</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1222,7 +1206,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1998-07-05 00:00:00</t>
+          <t>2000-03-11 00:00:00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1265,7 +1249,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2000-04-25 00:00:00</t>
+          <t>1997-03-05 00:00:00</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1308,7 +1292,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1995-06-08 00:00:00</t>
+          <t>1998-01-10 00:00:00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1351,7 +1335,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2002-10-27 00:00:00</t>
+          <t>1996-01-13 00:00:00</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1394,7 +1378,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1990-11-23 00:00:00</t>
+          <t>2003-03-02 00:00:00</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1437,7 +1421,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2001-10-16 00:00:00</t>
+          <t>1991-07-21 00:00:00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1480,7 +1464,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2003-09-20 00:00:00</t>
+          <t>1998-07-12 00:00:00</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1523,7 +1507,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1998-11-06 00:00:00</t>
+          <t>1994-08-14 00:00:00</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1566,7 +1550,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1997-11-14 00:00:00</t>
+          <t>1995-06-13 00:00:00</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1609,7 +1593,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1986-05-20 00:00:00</t>
+          <t>1995-06-08 00:00:00</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1652,7 +1636,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1999-01-29 00:00:00</t>
+          <t>1990-11-23 00:00:00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1695,7 +1679,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1999-06-23 00:00:00</t>
+          <t>2001-10-16 00:00:00</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1738,7 +1722,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>1997-01-19 00:00:00</t>
+          <t>2003-09-20 00:00:00</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1781,7 +1765,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1998-08-30 00:00:00</t>
+          <t>1998-11-06 00:00:00</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1824,7 +1808,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1999-03-14 00:00:00</t>
+          <t>1986-05-20 00:00:00</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1867,7 +1851,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1993-11-04 00:00:00</t>
+          <t>1999-01-29 00:00:00</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1910,7 +1894,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1998-06-13 00:00:00</t>
+          <t>1999-06-23 00:00:00</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1953,7 +1937,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1995-04-09 00:00:00</t>
+          <t>1997-01-19 00:00:00</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1996,7 +1980,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1999-05-25 00:00:00</t>
+          <t>1998-08-30 00:00:00</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2039,7 +2023,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2000-04-04 00:00:00</t>
+          <t>1999-03-14 00:00:00</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2057,22 +2041,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>"202606300060"</t>
+          <t>"202606300129"</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>"201808009"</t>
+          <t>"202208114"</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Produksi 2</t>
+          <t>HRGA</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2082,7 +2066,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1993-01-17 00:00:00</t>
+          <t>1993-11-04 00:00:00</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2093,29 +2077,29 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Ari Setya Budi</t>
+          <t>Arip Rahman</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>"202606300129"</t>
+          <t>"202606300060"</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>"202208114"</t>
+          <t>"201808009"</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>HRGA</t>
+          <t>Produksi 2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2125,7 +2109,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1994-09-04 00:00:00</t>
+          <t>1998-06-13 00:00:00</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2136,7 +2120,7 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Arip Rahman</t>
+          <t>Ari Setya Budi</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2152,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1985-02-26 00:00:00</t>
+          <t>1995-04-09 00:00:00</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2211,7 +2195,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1997-08-29 00:00:00</t>
+          <t>1999-05-25 00:00:00</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2254,7 +2238,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1997-01-11 00:00:00</t>
+          <t>2000-04-04 00:00:00</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2297,7 +2281,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1996-02-19 00:00:00</t>
+          <t>1993-01-17 00:00:00</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2340,7 +2324,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>1996-05-25 00:00:00</t>
+          <t>1985-02-26 00:00:00</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2383,7 +2367,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1999-09-10 00:00:00</t>
+          <t>1997-08-29 00:00:00</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2426,7 +2410,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2004-12-02 00:00:00</t>
+          <t>1997-01-11 00:00:00</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2469,7 +2453,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2000-02-03 00:00:00</t>
+          <t>1996-02-19 00:00:00</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2512,7 +2496,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1997-10-04 00:00:00</t>
+          <t>1996-05-25 00:00:00</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2555,7 +2539,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1990-09-19 00:00:00</t>
+          <t>1999-09-10 00:00:00</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2598,7 +2582,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>1998-07-14 00:00:00</t>
+          <t>2004-12-02 00:00:00</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2641,7 +2625,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2002-03-03 00:00:00</t>
+          <t>2000-02-03 00:00:00</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2684,7 +2668,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>1991-10-31 00:00:00</t>
+          <t>1997-10-04 00:00:00</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2727,7 +2711,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>1990-12-23 00:00:00</t>
+          <t>1990-09-19 00:00:00</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2770,7 +2754,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2001-02-13 00:00:00</t>
+          <t>2002-03-03 00:00:00</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2813,7 +2797,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2002-11-27 00:00:00</t>
+          <t>1998-07-14 00:00:00</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2856,7 +2840,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2001-05-31 00:00:00</t>
+          <t>1991-10-31 00:00:00</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2899,7 +2883,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2005-06-07 00:00:00</t>
+          <t>1990-12-23 00:00:00</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2942,7 +2926,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1996-09-29 00:00:00</t>
+          <t>2001-02-13 00:00:00</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2985,7 +2969,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>1998-05-17 00:00:00</t>
+          <t>2002-11-27 00:00:00</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3028,7 +3012,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1996-11-15 00:00:00</t>
+          <t>2005-06-07 00:00:00</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3069,7 +3053,11 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2001-05-31 00:00:00</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr">
         <is>
           <t>2026-07-06 00:00:00</t>
@@ -3110,7 +3098,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>1998-06-27 00:00:00</t>
+          <t>1996-09-29 00:00:00</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3196,7 +3184,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>1994-10-25 00:00:00</t>
+          <t>1998-05-17 00:00:00</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3239,7 +3227,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>1986-03-03 00:00:00</t>
+          <t>1998-06-27 00:00:00</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3282,7 +3270,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2001-02-05 00:00:00</t>
+          <t>1994-10-25 00:00:00</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3325,7 +3313,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-12-12 00:00:00</t>
+          <t>2001-02-05 00:00:00</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3368,7 +3356,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>1985-04-30 00:00:00</t>
+          <t>1986-03-03 00:00:00</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3411,7 +3399,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>1995-12-07 00:00:00</t>
+          <t>2026-12-12 00:00:00</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3454,7 +3442,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2001-08-27 00:00:00</t>
+          <t>1985-04-30 00:00:00</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3497,7 +3485,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>1998-10-05 00:00:00</t>
+          <t>1995-12-07 00:00:00</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3540,7 +3528,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2000-10-20 00:00:00</t>
+          <t>2001-08-27 00:00:00</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3583,7 +3571,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>1987-11-17 00:00:00</t>
+          <t>1998-10-05 00:00:00</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3626,7 +3614,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>1982-07-17 00:00:00</t>
+          <t>2000-10-20 00:00:00</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3669,7 +3657,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>1999-02-05 00:00:00</t>
+          <t>1987-11-17 00:00:00</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3712,7 +3700,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>1997-10-02 00:00:00</t>
+          <t>1982-07-17 00:00:00</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3755,7 +3743,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>1973-01-03 00:00:00</t>
+          <t>1999-02-05 00:00:00</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3798,7 +3786,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2000-03-03 00:00:00</t>
+          <t>1997-10-02 00:00:00</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3841,7 +3829,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>1989-07-05 00:00:00</t>
+          <t>1987-10-21 00:00:00</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3884,7 +3872,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>1987-10-21 00:00:00</t>
+          <t>1998-05-13 00:00:00</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3927,7 +3915,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>1986-07-12 00:00:00</t>
+          <t>2000-09-14 00:00:00</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3970,7 +3958,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>1998-05-13 00:00:00</t>
+          <t>1973-01-03 00:00:00</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4013,7 +4001,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2000-09-14 00:00:00</t>
+          <t>2000-03-03 00:00:00</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4056,7 +4044,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>1999-06-12 00:00:00</t>
+          <t>1986-07-12 00:00:00</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4099,7 +4087,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>1980-04-26 00:00:00</t>
+          <t>1989-07-05 00:00:00</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4142,7 +4130,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>1996-11-04 00:00:00</t>
+          <t>1999-06-12 00:00:00</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4185,7 +4173,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>1975-12-18 00:00:00</t>
+          <t>1980-04-26 00:00:00</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4228,7 +4216,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>1998-02-09 00:00:00</t>
+          <t>1996-11-04 00:00:00</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4271,7 +4259,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>1994-02-05 00:00:00</t>
+          <t>1975-12-18 00:00:00</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4314,7 +4302,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2000-03-31 00:00:00</t>
+          <t>1998-02-09 00:00:00</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4357,7 +4345,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>1988-04-03 00:00:00</t>
+          <t>1994-02-05 00:00:00</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4400,7 +4388,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>1997-03-29 00:00:00</t>
+          <t>2000-03-31 00:00:00</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4443,7 +4431,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>1989-08-31 00:00:00</t>
+          <t>1988-04-03 00:00:00</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4486,7 +4474,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2001-09-23 00:00:00</t>
+          <t>1997-03-29 00:00:00</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4529,7 +4517,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>1972-01-22 00:00:00</t>
+          <t>1989-08-31 00:00:00</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4572,7 +4560,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>1993-04-26 00:00:00</t>
+          <t>2001-09-23 00:00:00</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4615,7 +4603,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2000-06-30 00:00:00</t>
+          <t>1972-01-22 00:00:00</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4658,7 +4646,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2000-02-12 00:00:00</t>
+          <t>1993-04-26 00:00:00</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4701,7 +4689,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>1984-03-25 00:00:00</t>
+          <t>2000-06-30 00:00:00</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -4744,7 +4732,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2002-04-08 00:00:00</t>
+          <t>2000-02-12 00:00:00</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -4787,7 +4775,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>1999-10-29 00:00:00</t>
+          <t>1984-03-25 00:00:00</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4830,7 +4818,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2002-06-19 00:00:00</t>
+          <t>2002-04-08 00:00:00</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4873,7 +4861,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2003-04-05 00:00:00</t>
+          <t>1999-10-29 00:00:00</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4916,7 +4904,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2002-03-17 00:00:00</t>
+          <t>2002-06-19 00:00:00</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4959,7 +4947,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2003-08-17 00:00:00</t>
+          <t>2003-04-05 00:00:00</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -5002,7 +4990,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>1997-03-29 00:00:00</t>
+          <t>2002-03-17 00:00:00</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -5045,7 +5033,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>1988-05-28 00:00:00</t>
+          <t>2003-08-17 00:00:00</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -5088,7 +5076,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>1981-06-01 00:00:00</t>
+          <t>1997-03-29 00:00:00</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -5131,7 +5119,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>1993-06-19 00:00:00</t>
+          <t>2002-02-21 00:00:00</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -5174,7 +5162,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>1994-03-19 00:00:00</t>
+          <t>1999-11-20 00:00:00</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -5217,7 +5205,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>1995-12-28 00:00:00</t>
+          <t>1997-10-26 00:00:00</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -5260,7 +5248,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2002-02-21 00:00:00</t>
+          <t>2001-03-26 00:00:00</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -5303,7 +5291,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>1999-11-20 00:00:00</t>
+          <t>1988-05-28 00:00:00</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -5346,7 +5334,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2004-04-07 00:00:00</t>
+          <t>1981-06-01 00:00:00</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -5389,7 +5377,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>1998-08-30 00:00:00</t>
+          <t>1993-06-19 00:00:00</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -5432,7 +5420,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>1997-10-26 00:00:00</t>
+          <t>1995-12-28 00:00:00</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -5475,7 +5463,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>1995-12-12 00:00:00</t>
+          <t>2004-04-07 00:00:00</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -5518,7 +5506,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2001-03-26 00:00:00</t>
+          <t>1998-08-30 00:00:00</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -5561,7 +5549,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>1997-09-13 00:00:00</t>
+          <t>1995-12-12 00:00:00</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -5604,7 +5592,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>1995-01-14 00:00:00</t>
+          <t>1997-09-13 00:00:00</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -5647,7 +5635,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>1990-04-14 00:00:00</t>
+          <t>2003-01-07 00:00:00</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -5690,7 +5678,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2003-01-07 00:00:00</t>
+          <t>1990-04-14 00:00:00</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -5733,7 +5721,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>1998-04-28 00:00:00</t>
+          <t>2001-10-21 00:00:00</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -5776,7 +5764,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2001-10-21 00:00:00</t>
+          <t>1997-05-27 00:00:00</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -5819,7 +5807,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>1997-05-27 00:00:00</t>
+          <t>2000-07-18 00:00:00</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -5862,7 +5850,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2000-07-18 00:00:00</t>
+          <t>1979-10-23 00:00:00</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5905,7 +5893,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>1979-10-23 00:00:00</t>
+          <t>2001-12-13 00:00:00</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -5948,7 +5936,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2001-12-13 00:00:00</t>
+          <t>2002-05-21 00:00:00</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -5991,7 +5979,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2002-05-21 00:00:00</t>
+          <t>1996-10-20 00:00:00</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -6034,7 +6022,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>1996-10-20 00:00:00</t>
+          <t>2000-02-13 00:00:00</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -6077,7 +6065,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2000-02-13 00:00:00</t>
+          <t>1976-09-11 00:00:00</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -6120,7 +6108,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>1976-09-11 00:00:00</t>
+          <t>1997-05-20 00:00:00</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -6163,7 +6151,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>1997-05-20 00:00:00</t>
+          <t>1983-09-09 00:00:00</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -6206,7 +6194,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>1992-01-23 00:00:00</t>
+          <t>1988-10-27 00:00:00</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -6249,7 +6237,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2004-09-14 00:00:00</t>
+          <t>1992-01-23 00:00:00</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -6292,7 +6280,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>1983-09-09 00:00:00</t>
+          <t>2004-09-14 00:00:00</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -6378,7 +6366,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>1988-10-27 00:00:00</t>
+          <t>1988-07-06 00:00:00</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -6421,7 +6409,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>1988-07-06 00:00:00</t>
+          <t>1998-08-23 00:00:00</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -6464,7 +6452,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>1998-08-23 00:00:00</t>
+          <t>1998-02-25 00:00:00</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -6507,7 +6495,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>1998-02-25 00:00:00</t>
+          <t>2003-06-20 00:00:00</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -6550,7 +6538,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2003-06-20 00:00:00</t>
+          <t>2002-02-04 00:00:00</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -6593,7 +6581,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2002-02-04 00:00:00</t>
+          <t>2001-11-14 00:00:00</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -6636,7 +6624,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2001-11-14 00:00:00</t>
+          <t>1988-05-04 00:00:00</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -6722,7 +6710,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>1988-05-04 00:00:00</t>
+          <t>1999-08-12 00:00:00</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -6765,7 +6753,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>1999-08-12 00:00:00</t>
+          <t>1990-03-27 00:00:00</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -6808,7 +6796,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>1998-09-09 00:00:00</t>
+          <t>1994-03-04 00:00:00</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -6826,17 +6814,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>149</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>"202606300218"</t>
+          <t>"202606300462"</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>"202605120"</t>
+          <t>"202208110"</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -6851,7 +6839,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>1994-03-04 00:00:00</t>
+          <t>1992-04-12 00:00:00</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -6862,29 +6850,29 @@
       <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr">
         <is>
-          <t>M. RASYID SIDIK</t>
+          <t>Mafi Ridwan</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>"202606300462"</t>
+          <t>"202606300399"</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>"202208110"</t>
+          <t>"3215182709010000"</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Produksi 1</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6894,7 +6882,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>1990-03-27 00:00:00</t>
+          <t>2000-05-13 00:00:00</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -6905,29 +6893,29 @@
       <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Mafi Ridwan</t>
+          <t>MANTA CAHYANA</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>151</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>"202606300399"</t>
+          <t>"202606300074"</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>"3215182709010000"</t>
+          <t>"201306002"</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Produksi 1</t>
+          <t>Produksi 3</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6937,7 +6925,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>1994-07-04 00:00:00</t>
+          <t>1998-12-22 00:00:00</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6948,39 +6936,39 @@
       <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr">
         <is>
-          <t>MANTA CAHYANA</t>
+          <t>Mastur Hidayat</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>"202606300074"</t>
+          <t>"202606300122"</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>"201306002"</t>
+          <t>"202407038"</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Produksi 3</t>
+          <t>Produksi 2</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2001-09-27 00:00:00</t>
+          <t>1981-08-06 00:00:00</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -6991,39 +6979,39 @@
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Mastur Hidayat</t>
+          <t>MEIDRIANA ALIFA FITRI</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>153</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>"202606300122"</t>
+          <t>"202606300444"</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>"202407038"</t>
+          <t>"202207099"</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Produksi 2</t>
+          <t>Produksi 3</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>1992-04-12 00:00:00</t>
+          <t>1999-08-24 00:00:00</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -7034,29 +7022,29 @@
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
-          <t>MEIDRIANA ALIFA FITRI</t>
+          <t>Meifakur Satria Efendi</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>"202606300444"</t>
+          <t>"202606300288"</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>"202207099"</t>
+          <t>"23012334"</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Produksi 3</t>
+          <t>Supporting</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -7066,7 +7054,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2000-05-13 00:00:00</t>
+          <t>2002-01-07 00:00:00</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -7077,29 +7065,29 @@
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Meifakur Satria Efendi</t>
+          <t>MOCH ARSAD</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>155</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>"202606300288"</t>
+          <t>"202606300097"</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>"23012334"</t>
+          <t>"202204061"</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Supporting</t>
+          <t>Produksi 3</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -7109,7 +7097,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2002-05-13 00:00:00</t>
+          <t>1994-07-04 00:00:00</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -7120,29 +7108,29 @@
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
         <is>
-          <t>MOCH ARSAD</t>
+          <t>Mohamad Ramadhan</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>156</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>"202606300097"</t>
+          <t>"202606300373"</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>"202204061"</t>
+          <t>"24072695"</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Produksi 3</t>
+          <t>Supporting</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -7152,7 +7140,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>1993-08-02 00:00:00</t>
+          <t>1996-08-19 00:00:00</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -7163,29 +7151,29 @@
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Mohamad Ramadhan</t>
+          <t>MOHAMMAD ASEP RAMDHONI</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>"202606300373"</t>
+          <t>"202606300218"</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>"24072695"</t>
+          <t>"202605120"</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Supporting</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -7195,7 +7183,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>1998-12-22 00:00:00</t>
+          <t>1995-10-14 00:00:00</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -7206,7 +7194,7 @@
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
         <is>
-          <t>MOHAMMAD ASEP RAMDHONI</t>
+          <t>M. RASYID SIDIK</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7226,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>1981-08-06 00:00:00</t>
+          <t>1994-07-04 00:00:00</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -7281,7 +7269,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>1999-08-24 00:00:00</t>
+          <t>2001-09-27 00:00:00</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -7324,7 +7312,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2002-01-07 00:00:00</t>
+          <t>2002-05-13 00:00:00</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -7367,7 +7355,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2002-05-07 00:00:00</t>
+          <t>1993-08-02 00:00:00</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -7410,7 +7398,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>1994-07-04 00:00:00</t>
+          <t>2002-05-07 00:00:00</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -7453,7 +7441,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>1996-08-19 00:00:00</t>
+          <t>1998-01-05 00:00:00</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -7496,7 +7484,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>1998-01-05 00:00:00</t>
+          <t>1995-09-20 00:00:00</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -7539,7 +7527,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>1995-10-14 00:00:00</t>
+          <t>1993-10-06 00:00:00</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -7582,7 +7570,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>1995-09-20 00:00:00</t>
+          <t>1988-02-28 00:00:00</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -7625,7 +7613,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>1988-02-28 00:00:00</t>
+          <t>1999-11-08 00:00:00</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -7668,7 +7656,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>1999-11-08 00:00:00</t>
+          <t>1980-10-10 00:00:00</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -7711,7 +7699,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>1980-10-10 00:00:00</t>
+          <t>2000-01-16 00:00:00</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -7754,7 +7742,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2000-01-16 00:00:00</t>
+          <t>1998-07-29 00:00:00</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -7797,7 +7785,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>1993-10-06 00:00:00</t>
+          <t>2001-01-12 00:00:00</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -7840,7 +7828,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>1998-07-29 00:00:00</t>
+          <t>1997-07-23 00:00:00</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -7883,7 +7871,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2001-01-12 00:00:00</t>
+          <t>1996-11-18 00:00:00</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -7926,7 +7914,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>1997-07-23 00:00:00</t>
+          <t>1994-12-11 00:00:00</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -7969,7 +7957,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>1996-11-18 00:00:00</t>
+          <t>2002-05-15 00:00:00</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -8012,7 +8000,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>1994-12-11 00:00:00</t>
+          <t>1994-05-30 00:00:00</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -8055,7 +8043,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>2002-05-15 00:00:00</t>
+          <t>1992-08-15 00:00:00</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -8098,7 +8086,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>1994-05-30 00:00:00</t>
+          <t>1978-07-24 00:00:00</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -8141,7 +8129,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>1992-08-15 00:00:00</t>
+          <t>1983-07-15 00:00:00</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -8184,7 +8172,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>1978-07-24 00:00:00</t>
+          <t>2003-01-17 00:00:00</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -8227,7 +8215,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>1983-07-15 00:00:00</t>
+          <t>1998-03-01 00:00:00</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -8270,7 +8258,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>1996-08-02 00:00:00</t>
+          <t>1999-01-24 00:00:00</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -8313,7 +8301,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2003-01-17 00:00:00</t>
+          <t>1996-08-02 00:00:00</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -8399,7 +8387,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>1998-03-01 00:00:00</t>
+          <t>2002-09-14 00:00:00</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -8442,7 +8430,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>1999-01-24 00:00:00</t>
+          <t>1974-07-12 00:00:00</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -8485,7 +8473,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>2002-09-14 00:00:00</t>
+          <t>2000-07-26 00:00:00</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -8503,22 +8491,22 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>188</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>"202606300228"</t>
+          <t>"202606300386"</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>"202305041"</t>
+          <t>"202504102"</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Produksi 1</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -8528,7 +8516,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>2002-08-12 00:00:00</t>
+          <t>1993-12-19 00:00:00</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -8539,39 +8527,39 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>R. MUFTY JUSTIAWAN</t>
+          <t>RADEN FARHAN BEY DANUSAPUTRA</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>189</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>"202606300386"</t>
+          <t>"202606300433"</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>"202504102"</t>
+          <t>"202203052"</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Produksi 3</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>1974-07-12 00:00:00</t>
+          <t>1996-04-25 00:00:00</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -8582,24 +8570,24 @@
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>RADEN FARHAN BEY DANUSAPUTRA</t>
+          <t>RAFHIKA KHOIRIATULKAMALLIA</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>190</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>"202606300433"</t>
+          <t>"202606300285"</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>"202203052"</t>
+          <t>"202304032"</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -8612,7 +8600,11 @@
           <t>Perempuan</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>2002-08-12 00:00:00</t>
+        </is>
+      </c>
       <c r="G191" t="inlineStr">
         <is>
           <t>2026-06-30 00:00:00</t>
@@ -8621,39 +8613,39 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>RAFHIKA KHOIRIATULKAMALLIA</t>
+          <t>Rafika Nur Wahdah Purba</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>191</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>"202606300285"</t>
+          <t>"202606300226"</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>"202304032"</t>
+          <t>"202406033"</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Produksi 3</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>2000-07-26 00:00:00</t>
+          <t>1993-01-20 00:00:00</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -8664,39 +8656,39 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Rafika Nur Wahdah Purba</t>
+          <t>Rafly Fitipaldy</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>192</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>"202606300226"</t>
+          <t>"202606300298"</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>"202406033"</t>
+          <t>"23062491"</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Supporting</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>1998-07-03 00:00:00</t>
+          <t>1999-12-12 00:00:00</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -8707,39 +8699,39 @@
       <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Rafly Fitipaldy</t>
+          <t>RAHMA TIARA</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>193</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>"202606300298"</t>
+          <t>"202606300419"</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>"23062491"</t>
+          <t>"3215130407980000"</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Supporting</t>
+          <t>Produksi 2</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>1997-12-22 00:00:00</t>
+          <t>1989-04-24 00:00:00</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -8750,29 +8742,29 @@
       <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>RAHMA TIARA</t>
+          <t>RANDI AWALUDIN</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>194</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>"202606300419"</t>
+          <t>"202606300077"</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>"3215130407980000"</t>
+          <t>"3215171507020030"</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Produksi 2</t>
+          <t>Produksi 3</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -8782,7 +8774,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>2004-05-17 00:00:00</t>
+          <t>1998-07-26 00:00:00</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -8793,29 +8785,29 @@
       <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr">
         <is>
-          <t>RANDI AWALUDIN</t>
+          <t>RASJA RUDIANSYAH</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>195</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>"202606300077"</t>
+          <t>"202606300179"</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>"3215171507020030"</t>
+          <t>"202408048"</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Produksi 3</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -8825,7 +8817,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>1998-07-04 00:00:00</t>
+          <t>1998-07-03 00:00:00</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -8836,39 +8828,39 @@
       <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
-          <t>RASJA RUDIANSYAH</t>
+          <t>RASTA DIAN MAULA</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>196</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>"202606300179"</t>
+          <t>"202606300188"</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>"202408048"</t>
+          <t>"3173087005781000"</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Quality Control</t>
+          <t>RND</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>2002-07-15 00:00:00</t>
+          <t>1997-12-22 00:00:00</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -8879,29 +8871,29 @@
       <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr">
         <is>
-          <t>RASTA DIAN MAULA</t>
+          <t>RATNA SETYANINGRUM</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>197</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>"202606300188"</t>
+          <t>"202606300089"</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>"3173087005781000"</t>
+          <t>"202504107"</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>RND</t>
+          <t>RND 2</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -8911,7 +8903,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>2002-05-13 00:00:00</t>
+          <t>2004-05-17 00:00:00</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -8922,39 +8914,39 @@
       <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr">
         <is>
-          <t>RATNA SETYANINGRUM</t>
+          <t>RATRI DWIBUDANINGSIH</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>198</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>"202606300089"</t>
+          <t>"202606300335"</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>"202504107"</t>
+          <t>"202207091"</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>RND 2</t>
+          <t>Produksi 2</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>1978-05-30 00:00:00</t>
+          <t>1998-07-04 00:00:00</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -8965,39 +8957,39 @@
       <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
-          <t>RATRI DWIBUDANINGSIH</t>
+          <t>Reno Purnaya</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>199</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>"202606300335"</t>
+          <t>"202606300394"</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>"202207091"</t>
+          <t>"200609001"</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Produksi 2</t>
+          <t>Produksi 1</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>1986-11-26 00:00:00</t>
+          <t>2002-07-15 00:00:00</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -9008,39 +9000,39 @@
       <c r="H200" t="inlineStr"/>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Reno Purnaya</t>
+          <t>Retno Sri Marhaeni</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>200</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>"202606300394"</t>
+          <t>"202606300219"</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>"200609001"</t>
+          <t>"201904002"</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Produksi 1</t>
+          <t>Accounting</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>1993-12-19 00:00:00</t>
+          <t>2002-05-13 00:00:00</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -9051,29 +9043,29 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Retno Sri Marhaeni</t>
+          <t>Ridial Efendi</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>"202606300219"</t>
+          <t>"202606300303"</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>"201904002"</t>
+          <t>"202202040"</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Accounting</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -9083,7 +9075,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>1978-09-15 00:00:00</t>
+          <t>1978-05-30 00:00:00</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -9094,24 +9086,24 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Ridial Efendi</t>
+          <t>Rifki Aziz</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>202</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>"202606300303"</t>
+          <t>"202606300320"</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>"202202040"</t>
+          <t>"3214030903010000"</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -9126,7 +9118,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>1996-07-09 00:00:00</t>
+          <t>1986-11-26 00:00:00</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -9137,29 +9129,29 @@
       <c r="H203" t="inlineStr"/>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Rifki Aziz</t>
+          <t>RIFQI RYAN FADILLAH</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>203</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>"202606300320"</t>
+          <t>"202606300389"</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>"3214030903010000"</t>
+          <t>"202211130"</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -9169,7 +9161,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>1998-11-17 00:00:00</t>
+          <t>1978-09-15 00:00:00</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -9180,39 +9172,39 @@
       <c r="H204" t="inlineStr"/>
       <c r="I204" t="inlineStr">
         <is>
-          <t>RIFQI RYAN FADILLAH</t>
+          <t>Riki Anggi Putra</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>204</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>"202606300389"</t>
+          <t>"202606300321"</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>"202211130"</t>
+          <t>"200601001"</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Laki-laki</t>
+          <t>Perempuan</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2001-03-09 00:00:00</t>
+          <t>1996-07-09 00:00:00</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -9223,39 +9215,39 @@
       <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Riki Anggi Putra</t>
+          <t>Rini Susilowati</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>205</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>"202606300321"</t>
+          <t>"202606300243"</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>"200601001"</t>
+          <t>"201805010"</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Produksi 1</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>1999-10-21 00:00:00</t>
+          <t>1998-11-17 00:00:00</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -9266,29 +9258,29 @@
       <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Rini Susilowati</t>
+          <t>Ripal Sadar Pamungkas</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>206</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>"202606300243"</t>
+          <t>"202606300067"</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>"201805010"</t>
+          <t>"202001077"</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Produksi 1</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -9298,7 +9290,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>1986-03-26 00:00:00</t>
+          <t>2001-03-09 00:00:00</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -9309,29 +9301,29 @@
       <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Ripal Sadar Pamungkas</t>
+          <t>Riyan Ropi Fauzi</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>207</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>"202606300067"</t>
+          <t>"202606300383"</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>"202001077"</t>
+          <t>"202404016"</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -9341,7 +9333,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>1996-04-25 00:00:00</t>
+          <t>1999-10-21 00:00:00</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -9352,24 +9344,24 @@
       <c r="H208" t="inlineStr"/>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Riyan Ropi Fauzi</t>
+          <t>Rizal Fatoni</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>208</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>"202606300383"</t>
+          <t>"202606300223"</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>"202404016"</t>
+          <t>"3215141208020000"</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -9384,7 +9376,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>1995-01-07 00:00:00</t>
+          <t>1986-03-26 00:00:00</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -9395,29 +9387,29 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Rizal Fatoni</t>
+          <t>RIZKY ARDIANSYAH SOLIHIN</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>209</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>"202606300223"</t>
+          <t>"202606300228"</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>"3215141208020000"</t>
+          <t>"202305041"</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>Produksi 1</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -9427,7 +9419,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>1996-04-08 00:00:00</t>
+          <t>1995-01-07 00:00:00</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -9438,7 +9430,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>RIZKY ARDIANSYAH SOLIHIN</t>
+          <t>R. MUFTY JUSTIAWAN</t>
         </is>
       </c>
     </row>
@@ -9470,7 +9462,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>1993-01-20 00:00:00</t>
+          <t>1996-04-08 00:00:00</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -9513,7 +9505,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>1999-12-12 00:00:00</t>
+          <t>1983-03-16 00:00:00</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -9556,7 +9548,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>1989-04-24 00:00:00</t>
+          <t>1998-11-26 00:00:00</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -9599,7 +9591,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>1983-03-16 00:00:00</t>
+          <t>1999-08-21 00:00:00</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -9642,7 +9634,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>1998-07-26 00:00:00</t>
+          <t>2002-04-19 00:00:00</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -9685,7 +9677,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>2001-04-12 00:00:00</t>
+          <t>1995-05-31 00:00:00</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -9728,7 +9720,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>1984-08-28 00:00:00</t>
+          <t>2000-09-23 00:00:00</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -9771,7 +9763,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>1998-11-26 00:00:00</t>
+          <t>1992-04-04 00:00:00</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -9814,7 +9806,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>1995-09-29 00:00:00</t>
+          <t>1996-11-10 00:00:00</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -9857,7 +9849,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>1998-10-07 00:00:00</t>
+          <t>1997-06-28 00:00:00</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -9900,7 +9892,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>1999-08-21 00:00:00</t>
+          <t>1996-08-08 00:00:00</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -9943,7 +9935,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>1978-09-09 00:00:00</t>
+          <t>1992-03-15 00:00:00</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -9986,7 +9978,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>1995-09-04 00:00:00</t>
+          <t>1997-04-30 00:00:00</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -10029,7 +10021,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>1999-05-25 00:00:00</t>
+          <t>2001-04-12 00:00:00</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -10072,7 +10064,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>1996-11-10 00:00:00</t>
+          <t>1984-08-28 00:00:00</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -10115,7 +10107,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2001-05-26 00:00:00</t>
+          <t>1995-09-29 00:00:00</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -10158,7 +10150,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>1989-09-04 00:00:00</t>
+          <t>1998-10-07 00:00:00</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -10201,7 +10193,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>2002-04-19 00:00:00</t>
+          <t>1978-09-09 00:00:00</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -10244,7 +10236,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>1999-06-09 00:00:00</t>
+          <t>1995-09-04 00:00:00</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -10287,7 +10279,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>1974-07-26 00:00:00</t>
+          <t>1999-05-25 00:00:00</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -10330,7 +10322,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>1995-05-31 00:00:00</t>
+          <t>1996-11-10 00:00:00</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -10373,7 +10365,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>1997-11-07 00:00:00</t>
+          <t>2001-05-26 00:00:00</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -10416,7 +10408,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2000-09-23 00:00:00</t>
+          <t>1989-09-04 00:00:00</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -10459,7 +10451,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>1993-09-02 00:00:00</t>
+          <t>1999-06-09 00:00:00</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -10502,7 +10494,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>2000-10-05 00:00:00</t>
+          <t>1974-07-26 00:00:00</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -10545,7 +10537,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>1975-07-14 00:00:00</t>
+          <t>1997-11-07 00:00:00</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -10588,7 +10580,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>1992-04-04 00:00:00</t>
+          <t>1993-09-02 00:00:00</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -10631,7 +10623,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>1996-11-10 00:00:00</t>
+          <t>2000-10-05 00:00:00</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -10674,7 +10666,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>1999-07-28 00:00:00</t>
+          <t>1975-07-14 00:00:00</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -10717,7 +10709,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>1993-08-29 00:00:00</t>
+          <t>1999-07-28 00:00:00</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -10760,7 +10752,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>1996-04-11 00:00:00</t>
+          <t>1993-08-29 00:00:00</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -10803,7 +10795,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>1990-09-19 00:00:00</t>
+          <t>1996-04-11 00:00:00</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -10846,7 +10838,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>1997-06-28 00:00:00</t>
+          <t>1990-09-19 00:00:00</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -10932,7 +10924,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>1996-08-08 00:00:00</t>
+          <t>2001-08-28 00:00:00</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -10975,7 +10967,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>1992-03-15 00:00:00</t>
+          <t>1987-05-14 00:00:00</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -11016,7 +11008,11 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>2001-03-13 00:00:00</t>
+        </is>
+      </c>
       <c r="G247" t="inlineStr">
         <is>
           <t>2026-07-06 00:00:00</t>
@@ -11057,7 +11053,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>2001-08-28 00:00:00</t>
+          <t>2000-09-08 00:00:00</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -11100,7 +11096,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>1997-04-30 00:00:00</t>
+          <t>1994-08-04 00:00:00</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -11186,7 +11182,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>2001-03-13 00:00:00</t>
+          <t>1988-05-02 00:00:00</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -11229,7 +11225,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>2000-09-08 00:00:00</t>
+          <t>1989-08-02 00:00:00</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -11272,7 +11268,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>1994-08-04 00:00:00</t>
+          <t>1994-04-26 00:00:00</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -11315,7 +11311,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>1987-05-14 00:00:00</t>
+          <t>1994-08-07 00:00:00</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -11333,22 +11329,22 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>254</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>"202606300407"</t>
+          <t>"202606300143"</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>"202204065"</t>
+          <t>"201211001"</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Produksi 2</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -11358,7 +11354,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>1989-08-02 00:00:00</t>
+          <t>1971-03-16 00:00:00</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -11369,29 +11365,29 @@
       <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Tri Riswanto</t>
+          <t>TRIONO SAPUTRO</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>255</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>"202606300143"</t>
+          <t>"202606300407"</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>"201211001"</t>
+          <t>"202204065"</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Produksi 2</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -11401,7 +11397,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>1988-05-02 00:00:00</t>
+          <t>1982-03-23 00:00:00</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -11412,7 +11408,7 @@
       <c r="H256" t="inlineStr"/>
       <c r="I256" t="inlineStr">
         <is>
-          <t>TRIONO SAPUTRO</t>
+          <t>Tri Riswanto</t>
         </is>
       </c>
     </row>
@@ -11444,7 +11440,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>1994-04-26 00:00:00</t>
+          <t>1983-12-27 00:00:00</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -11487,7 +11483,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>1994-08-07 00:00:00</t>
+          <t>1996-01-20 00:00:00</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -11530,7 +11526,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>1971-03-16 00:00:00</t>
+          <t>2000-04-21 00:00:00</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -11573,7 +11569,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>1982-03-23 00:00:00</t>
+          <t>2000-07-22 00:00:00</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -11616,7 +11612,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>1983-12-27 00:00:00</t>
+          <t>2000-07-29 00:00:00</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -11659,7 +11655,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>1996-01-20 00:00:00</t>
+          <t>2000-01-18 00:00:00</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -11702,7 +11698,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>2000-04-21 00:00:00</t>
+          <t>1979-10-08 00:00:00</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -11745,7 +11741,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>2000-07-22 00:00:00</t>
+          <t>2000-03-20 00:00:00</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -11788,7 +11784,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2000-07-29 00:00:00</t>
+          <t>1999-07-09 00:00:00</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -11831,7 +11827,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>2000-01-18 00:00:00</t>
+          <t>1993-05-02 00:00:00</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -11874,7 +11870,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>1979-10-08 00:00:00</t>
+          <t>2000-10-29 00:00:00</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -11917,7 +11913,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>2000-03-20 00:00:00</t>
+          <t>2000-07-28 00:00:00</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -11960,7 +11956,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>1999-07-09 00:00:00</t>
+          <t>1991-07-11 00:00:00</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -12003,7 +11999,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>1991-07-11 00:00:00</t>
+          <t>1999-11-10 00:00:00</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -12046,7 +12042,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>1999-11-10 00:00:00</t>
+          <t>1996-01-25 00:00:00</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -12089,7 +12085,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>1996-01-25 00:00:00</t>
+          <t>1995-09-21 00:00:00</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -12132,7 +12128,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>1995-09-21 00:00:00</t>
+          <t>1995-05-20 00:00:00</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -12175,7 +12171,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>1993-05-02 00:00:00</t>
+          <t>1982-01-28 00:00:00</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -12216,7 +12212,11 @@
           <t>Laki-laki</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr"/>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>1988-07-23 00:00:00</t>
+        </is>
+      </c>
       <c r="G275" t="inlineStr">
         <is>
           <t>2026-07-07 00:00:00</t>
@@ -12257,7 +12257,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>2000-10-29 00:00:00</t>
+          <t>1996-11-15 00:00:00</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -12300,7 +12300,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>1995-05-20 00:00:00</t>
+          <t>1994-03-19 00:00:00</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>2000-07-28 00:00:00</t>
+          <t>1995-01-14 00:00:00</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>1982-01-28 00:00:00</t>
+          <t>1998-04-28 00:00:00</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -12429,7 +12429,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>1988-07-23 00:00:00</t>
+          <t>1998-09-09 00:00:00</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">

</xml_diff>